<commit_message>
Medication chart: Pawfolio note with QR code and site address on builder printouts, PDFs and spreadsheet
</commit_message>
<xml_diff>
--- a/pet-medication-chart/pet-medication-chart.xlsx
+++ b/pet-medication-chart/pet-medication-chart.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Week 1'!$A$1:$J$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Week 1'!$A$1:$J$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,6 +65,24 @@
       <color rgb="0001696F"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0012676E"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002B2723"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00555555"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -427,7 +445,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -602,6 +620,9 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -967,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1012,7 +1033,6 @@
       <c r="E3" s="34" t="n"/>
       <c r="F3" s="27" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
@@ -1273,11 +1293,31 @@
       <c r="I17" s="67" t="n"/>
       <c r="J17" s="67" t="n"/>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>"Due" = next scheduled time.   "Taken" = time the dose was actually given.   ↓ next box is below, → next box is the same row in the next day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="70" t="inlineStr">
+        <is>
+          <t>Get free dose reminders on your phone with Pawfolio Free. Using a sitter? Pawfolio Complete shares dose times and shows who gave each one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="71" t="inlineStr">
+        <is>
+          <t>cleartrackapps.com/pawfolio</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="72" t="inlineStr">
+        <is>
+          <t>Free chart from cleartrackapps.com/pet-medication-chart</t>
         </is>
       </c>
     </row>
@@ -1299,6 +1339,9 @@
     <mergeCell ref="B10:B13"/>
     <mergeCell ref="E3:F3"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId1"/>
+  </hyperlinks>
   <printOptions verticalCentered="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>

</xml_diff>